<commit_message>
Atualiza dados - 10/08/2026 22:31
</commit_message>
<xml_diff>
--- a/pat/PAT.xlsx
+++ b/pat/PAT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\pat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF349E5E-2D9B-421D-836C-97D81C2B8B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F4013BA-2B1D-4F54-A006-EE3AB2B5B03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenarios_hml" sheetId="1" r:id="rId1"/>
@@ -48,9 +48,6 @@
     <t>Cenário de teste</t>
   </si>
   <si>
-    <t xml:space="preserve">Status do teste </t>
-  </si>
-  <si>
     <t>Acionar Cumprimento de exigência de autodeclaração sem finalizar a autodeclaração</t>
   </si>
   <si>
@@ -1289,6 +1286,9 @@
   </si>
   <si>
     <t>Em Execução</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
 </sst>
 </file>
@@ -1826,16 +1826,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>57</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -1843,16 +1843,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -1860,16 +1860,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -1877,16 +1877,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -1894,16 +1894,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1911,16 +1911,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -1928,16 +1928,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -1945,16 +1945,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -1962,16 +1962,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -1979,16 +1979,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -1996,16 +1996,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2013,16 +2013,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2030,16 +2030,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2047,16 +2047,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2064,16 +2064,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -2081,16 +2081,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -2098,16 +2098,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
@@ -2115,16 +2115,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -2132,16 +2132,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2149,16 +2149,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2166,16 +2166,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2183,16 +2183,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -2200,16 +2200,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -2217,16 +2217,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -2234,16 +2234,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2251,16 +2251,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2268,16 +2268,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2285,16 +2285,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -2302,16 +2302,16 @@
         <v>28</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -2319,16 +2319,16 @@
         <v>29</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
@@ -2336,16 +2336,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
@@ -2353,16 +2353,16 @@
         <v>31</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
@@ -2370,16 +2370,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
@@ -2387,16 +2387,16 @@
         <v>33</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
@@ -2404,16 +2404,16 @@
         <v>34</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2421,16 +2421,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2438,16 +2438,16 @@
         <v>36</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -2455,14 +2455,14 @@
         <v>37</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
@@ -2470,14 +2470,14 @@
         <v>38</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C39" s="18" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
@@ -2485,14 +2485,14 @@
         <v>39</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C40" s="17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -2500,14 +2500,14 @@
         <v>40</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C41" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -2515,14 +2515,14 @@
         <v>41</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -2530,14 +2530,14 @@
         <v>42</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C43" s="20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D43" s="3"/>
       <c r="E43" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -2545,14 +2545,14 @@
         <v>43</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C44" s="20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
@@ -2655,34 +2655,34 @@
   <sheetData>
     <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="6" t="s">
         <v>18</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza dados - 13/08/2026  9:04
</commit_message>
<xml_diff>
--- a/pat/PAT.xlsx
+++ b/pat/PAT.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\pat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F4013BA-2B1D-4F54-A006-EE3AB2B5B03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA648C81-B135-494E-AEAD-3078B644054A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenarios_hml" sheetId="1" r:id="rId1"/>
     <sheet name="ResumoDiario" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Cenarios_hml!$A$1:$E$44</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="61">
   <si>
     <t>Número do cenário</t>
   </si>
@@ -1285,10 +1288,19 @@
     <t>Sim</t>
   </si>
   <si>
-    <t>Em Execução</t>
-  </si>
-  <si>
     <t>Status</t>
+  </si>
+  <si>
+    <t>Aprovado</t>
+  </si>
+  <si>
+    <t>Em Teste</t>
+  </si>
+  <si>
+    <t>Disponivel para reteste</t>
+  </si>
+  <si>
+    <t>Não Liberado</t>
   </si>
 </sst>
 </file>
@@ -1347,7 +1359,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1375,6 +1387,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
@@ -1420,7 +1456,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1430,9 +1466,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1458,9 +1491,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1474,6 +1504,57 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1811,12 +1892,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3CBE49E-44A1-44E6-BD58-CEAED8D0EF53}">
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.77734375" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="152.5546875" customWidth="1"/>
+    <col min="3" max="3" width="168.21875" customWidth="1"/>
     <col min="4" max="4" width="19.5546875" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24" style="2" bestFit="1" customWidth="1"/>
   </cols>
@@ -1832,211 +1913,211 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A2" s="3">
+      <c r="A2" s="19">
         <v>1</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="22">
+        <v>2</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A4" s="19">
+        <v>3</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A5" s="24">
+        <v>4</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" s="24" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="24">
+        <v>5</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="24" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A7" s="19">
         <v>6</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="14" t="s">
+      <c r="B7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
-        <v>3</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E4" s="3" t="s">
+      <c r="C7" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="E7" s="19" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
-        <v>4</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
-        <v>5</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
-        <v>6</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E7" s="3" t="s">
+    <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="24">
+        <v>7</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="33" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" s="24" t="s">
         <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="3">
-        <v>7</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="12" t="s">
         <v>27</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="3">
+      <c r="A10" s="24">
         <v>9</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>54</v>
+      <c r="D10" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="3">
+      <c r="A11" s="19">
         <v>10</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E11" s="3" t="s">
+      <c r="D11" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="E11" s="19" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="3">
+      <c r="A12" s="19">
         <v>11</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>54</v>
+      <c r="D12" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="E12" s="19" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>12</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>54</v>
@@ -2046,65 +2127,65 @@
       <c r="A14" s="3">
         <v>13</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="11" t="s">
         <v>32</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="3">
+    <row r="15" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="19">
         <v>14</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>54</v>
+      <c r="D15" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" s="19" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="3">
+      <c r="A16" s="24">
         <v>15</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>54</v>
+      <c r="D16" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="14" t="s">
         <v>3</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>54</v>
@@ -2114,48 +2195,48 @@
       <c r="A18" s="3">
         <v>17</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="15" t="s">
         <v>4</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="3">
+      <c r="A19" s="24">
         <v>18</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="16" t="s">
+      <c r="C19" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>54</v>
+      <c r="D19" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>19</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="12" t="s">
         <v>34</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>54</v>
@@ -2165,14 +2246,14 @@
       <c r="A21" s="3">
         <v>20</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="12" t="s">
         <v>35</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>54</v>
@@ -2182,14 +2263,14 @@
       <c r="A22" s="3">
         <v>21</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="12" t="s">
         <v>36</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>54</v>
@@ -2199,118 +2280,118 @@
       <c r="A23" s="3">
         <v>22</v>
       </c>
-      <c r="B23" s="14" t="s">
+      <c r="B23" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="12" t="s">
         <v>37</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="3">
+      <c r="A24" s="24">
         <v>23</v>
       </c>
-      <c r="B24" s="14" t="s">
+      <c r="B24" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>54</v>
+      <c r="D24" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E24" s="24" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A25" s="3">
+      <c r="A25" s="19">
         <v>24</v>
       </c>
-      <c r="B25" s="14" t="s">
+      <c r="B25" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E25" s="3" t="s">
+      <c r="D25" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" s="19" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="3">
+      <c r="A26" s="19">
         <v>25</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="3">
+      <c r="D26" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="E26" s="19" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A27" s="22">
         <v>26</v>
       </c>
-      <c r="B27" s="14" t="s">
+      <c r="B27" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E27" s="3" t="s">
+      <c r="D27" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E27" s="22" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="3">
+    <row r="28" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="22">
         <v>27</v>
       </c>
-      <c r="B28" s="14" t="s">
+      <c r="B28" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C28" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="D28" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E28" s="3" t="s">
+      <c r="D28" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="22" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="3">
+      <c r="A29" s="24">
         <v>28</v>
       </c>
-      <c r="B29" s="14" t="s">
+      <c r="B29" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="C29" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E29" s="3" t="s">
+      <c r="D29" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E29" s="24" t="s">
         <v>55</v>
       </c>
     </row>
@@ -2318,14 +2399,14 @@
       <c r="A30" s="3">
         <v>29</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="B30" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="C30" s="15" t="s">
         <v>3</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>54</v>
@@ -2335,14 +2416,14 @@
       <c r="A31" s="3">
         <v>30</v>
       </c>
-      <c r="B31" s="14" t="s">
+      <c r="B31" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C31" s="16" t="s">
+      <c r="C31" s="14" t="s">
         <v>3</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>54</v>
@@ -2352,130 +2433,134 @@
       <c r="A32" s="3">
         <v>31</v>
       </c>
-      <c r="B32" s="14" t="s">
+      <c r="B32" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C32" s="17" t="s">
+      <c r="C32" s="15" t="s">
         <v>43</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="3">
+    <row r="33" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="22">
         <v>32</v>
       </c>
-      <c r="B33" s="14" t="s">
+      <c r="B33" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C33" s="17" t="s">
+      <c r="C33" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="D33" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E33" s="3" t="s">
+      <c r="D33" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E33" s="22" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="3">
+      <c r="A34" s="22">
         <v>33</v>
       </c>
-      <c r="B34" s="14" t="s">
+      <c r="B34" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C34" s="17" t="s">
+      <c r="C34" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="D34" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E34" s="3" t="s">
+      <c r="D34" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E34" s="22" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A35" s="3">
+      <c r="A35" s="22">
         <v>34</v>
       </c>
-      <c r="B35" s="14" t="s">
+      <c r="B35" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C35" s="17" t="s">
+      <c r="C35" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="D35" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="D35" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E35" s="22" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>35</v>
       </c>
-      <c r="B36" s="14" t="s">
+      <c r="B36" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C36" s="19" t="s">
+      <c r="C36" s="17" t="s">
         <v>46</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>36</v>
       </c>
-      <c r="B37" s="14" t="s">
+      <c r="B37" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C37" s="19" t="s">
+      <c r="C37" s="17" t="s">
         <v>42</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A38" s="3">
+      <c r="A38" s="24">
         <v>37</v>
       </c>
-      <c r="B38" s="14" t="s">
+      <c r="B38" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="C38" s="20" t="s">
+      <c r="C38" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="D38" s="3"/>
-      <c r="E38" s="3" t="s">
-        <v>54</v>
+      <c r="D38" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E38" s="24" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>38</v>
       </c>
-      <c r="B39" s="14" t="s">
+      <c r="B39" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C39" s="18" t="s">
+      <c r="C39" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="D39" s="3"/>
+      <c r="D39" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="E39" s="3" t="s">
         <v>54</v>
       </c>
@@ -2484,13 +2569,15 @@
       <c r="A40" s="3">
         <v>39</v>
       </c>
-      <c r="B40" s="14" t="s">
+      <c r="B40" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C40" s="17" t="s">
+      <c r="C40" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="D40" s="3"/>
+      <c r="D40" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="E40" s="3" t="s">
         <v>54</v>
       </c>
@@ -2499,13 +2586,15 @@
       <c r="A41" s="3">
         <v>40</v>
       </c>
-      <c r="B41" s="14" t="s">
+      <c r="B41" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C41" s="20" t="s">
+      <c r="C41" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="D41" s="3"/>
+      <c r="D41" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="E41" s="3" t="s">
         <v>54</v>
       </c>
@@ -2514,13 +2603,15 @@
       <c r="A42" s="3">
         <v>41</v>
       </c>
-      <c r="B42" s="14" t="s">
+      <c r="B42" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C42" s="20" t="s">
+      <c r="C42" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="D42" s="3"/>
+      <c r="D42" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="E42" s="3" t="s">
         <v>54</v>
       </c>
@@ -2529,13 +2620,15 @@
       <c r="A43" s="3">
         <v>42</v>
       </c>
-      <c r="B43" s="14" t="s">
+      <c r="B43" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C43" s="20" t="s">
+      <c r="C43" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="D43" s="3"/>
+      <c r="D43" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="E43" s="3" t="s">
         <v>54</v>
       </c>
@@ -2544,95 +2637,21 @@
       <c r="A44" s="3">
         <v>43</v>
       </c>
-      <c r="B44" s="14" t="s">
+      <c r="B44" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C44" s="20" t="s">
+      <c r="C44" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="D44" s="3"/>
+      <c r="D44" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="E44" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A45" s="3"/>
-      <c r="B45" s="3"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="4"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A51" s="3"/>
-      <c r="B51" s="3"/>
-      <c r="C51" s="4"/>
-      <c r="D51" s="3"/>
-      <c r="E51" s="3"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A52" s="3"/>
-      <c r="B52" s="3"/>
-      <c r="C52" s="4"/>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A53" s="3"/>
-      <c r="B53" s="3"/>
-      <c r="C53" s="4"/>
-      <c r="D53" s="3"/>
-      <c r="E53" s="3"/>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="3"/>
-      <c r="B54" s="3"/>
-      <c r="C54" s="4"/>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A55" s="3"/>
-      <c r="B55" s="3"/>
-      <c r="C55" s="4"/>
-      <c r="D55" s="3"/>
-      <c r="E55" s="3"/>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:E44" xr:uid="{A3CBE49E-44A1-44E6-BD58-CEAED8D0EF53}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
@@ -2654,126 +2673,126 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="7">
+      <c r="A2" s="6">
         <v>0.41666666666666669</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="7">
         <v>46244</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="8">
         <v>0</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="8">
         <v>36</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="8">
         <v>0</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="8">
         <v>0</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="8">
         <v>0</v>
       </c>
-      <c r="H2" s="9">
+      <c r="H2" s="8">
         <v>0</v>
       </c>
-      <c r="I2" s="9">
+      <c r="I2" s="8">
         <v>0</v>
       </c>
-      <c r="J2" s="10">
+      <c r="J2" s="9">
         <f>C2+D2+E2+F2+G2+H2+I2</f>
         <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="7"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="10">
+      <c r="A3" s="6"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="9">
         <f t="shared" ref="J3:J6" si="0">C3+D3+E3+F3+G3+H3+I3</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="7"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="10">
+      <c r="A4" s="6"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="9">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="7"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="10">
+      <c r="A5" s="6"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="9">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="10">
+      <c r="A6" s="6"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="9">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Atualiza dados - 13/08/2026 10:52
</commit_message>
<xml_diff>
--- a/pat/PAT.xlsx
+++ b/pat/PAT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\pat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA648C81-B135-494E-AEAD-3078B644054A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A835902-C72A-4FE4-9EC6-0E149FC08DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenarios_hml" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="61">
   <si>
     <t>Número do cenário</t>
   </si>
@@ -84,16 +84,7 @@
     <t>Data</t>
   </si>
   <si>
-    <t>Pendente de cenário</t>
-  </si>
-  <si>
-    <t>Homologado com sucesso</t>
-  </si>
-  <si>
     <t>Reprovado</t>
-  </si>
-  <si>
-    <t>Aguardando Correção</t>
   </si>
   <si>
     <t>Disponível para reteste</t>
@@ -1301,6 +1292,15 @@
   </si>
   <si>
     <t>Não Liberado</t>
+  </si>
+  <si>
+    <t>Em Execução</t>
+  </si>
+  <si>
+    <t>Não Liberados</t>
+  </si>
+  <si>
+    <t>Aprovados</t>
   </si>
 </sst>
 </file>
@@ -1892,6 +1892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3CBE49E-44A1-44E6-BD58-CEAED8D0EF53}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1913,13 +1914,13 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="19">
         <v>1</v>
       </c>
@@ -1927,16 +1928,16 @@
         <v>9</v>
       </c>
       <c r="C2" s="31" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="22">
         <v>2</v>
       </c>
@@ -1944,16 +1945,16 @@
         <v>9</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19">
         <v>3</v>
       </c>
@@ -1961,16 +1962,16 @@
         <v>9</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="24">
         <v>4</v>
       </c>
@@ -1978,16 +1979,16 @@
         <v>9</v>
       </c>
       <c r="C5" s="30" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="24">
         <v>5</v>
       </c>
@@ -1995,16 +1996,16 @@
         <v>9</v>
       </c>
       <c r="C6" s="30" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="19">
         <v>6</v>
       </c>
@@ -2012,16 +2013,16 @@
         <v>9</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="24">
         <v>7</v>
       </c>
@@ -2029,13 +2030,13 @@
         <v>8</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -2046,16 +2047,16 @@
         <v>8</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="24">
         <v>9</v>
       </c>
@@ -2063,16 +2064,16 @@
         <v>8</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="19">
         <v>10</v>
       </c>
@@ -2080,16 +2081,16 @@
         <v>8</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="19">
         <v>11</v>
       </c>
@@ -2097,16 +2098,16 @@
         <v>8</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -2114,16 +2115,16 @@
         <v>8</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -2131,16 +2132,16 @@
         <v>8</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="19">
         <v>14</v>
       </c>
@@ -2148,16 +2149,16 @@
         <v>8</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="24">
         <v>15</v>
       </c>
@@ -2168,13 +2169,13 @@
         <v>2</v>
       </c>
       <c r="D16" s="24" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E16" s="24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -2185,13 +2186,13 @@
         <v>3</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -2202,13 +2203,13 @@
         <v>4</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="24">
         <v>18</v>
       </c>
@@ -2219,13 +2220,13 @@
         <v>5</v>
       </c>
       <c r="D19" s="24" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -2233,16 +2234,16 @@
         <v>8</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -2250,16 +2251,16 @@
         <v>8</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -2267,16 +2268,16 @@
         <v>8</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -2284,16 +2285,16 @@
         <v>8</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="24">
         <v>23</v>
       </c>
@@ -2301,50 +2302,50 @@
         <v>9</v>
       </c>
       <c r="C24" s="26" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D24" s="24" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="19">
         <v>24</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C25" s="29" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="19">
         <v>25</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="22">
         <v>26</v>
       </c>
@@ -2352,16 +2353,16 @@
         <v>8</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D27" s="22" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="22">
         <v>27</v>
       </c>
@@ -2369,33 +2370,33 @@
         <v>8</v>
       </c>
       <c r="C28" s="27" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D28" s="22" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E28" s="22" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="24">
         <v>28</v>
       </c>
       <c r="B29" s="25" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D29" s="24" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E29" s="24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -2406,13 +2407,13 @@
         <v>3</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -2423,13 +2424,13 @@
         <v>3</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -2437,16 +2438,16 @@
         <v>8</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="26.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="22">
         <v>32</v>
       </c>
@@ -2457,13 +2458,13 @@
         <v>5</v>
       </c>
       <c r="D33" s="22" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="22">
         <v>33</v>
       </c>
@@ -2471,16 +2472,16 @@
         <v>10</v>
       </c>
       <c r="C34" s="28" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D34" s="22" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E34" s="22" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="52.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="22">
         <v>34</v>
       </c>
@@ -2488,16 +2489,16 @@
         <v>10</v>
       </c>
       <c r="C35" s="28" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D35" s="22" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -2505,16 +2506,16 @@
         <v>10</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -2522,16 +2523,16 @@
         <v>10</v>
       </c>
       <c r="C37" s="17" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="24">
         <v>37</v>
       </c>
@@ -2539,16 +2540,16 @@
         <v>10</v>
       </c>
       <c r="C38" s="35" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D38" s="24" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E38" s="24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -2559,13 +2560,13 @@
         <v>3</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -2573,16 +2574,16 @@
         <v>10</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -2590,16 +2591,16 @@
         <v>10</v>
       </c>
       <c r="C41" s="18" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -2607,16 +2608,16 @@
         <v>8</v>
       </c>
       <c r="C42" s="18" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -2624,16 +2625,16 @@
         <v>8</v>
       </c>
       <c r="C43" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E43" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D43" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -2641,38 +2642,43 @@
         <v>8</v>
       </c>
       <c r="C44" s="18" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E44" xr:uid="{A3CBE49E-44A1-44E6-BD58-CEAED8D0EF53}"/>
+  <autoFilter ref="A1:E44" xr:uid="{A3CBE49E-44A1-44E6-BD58-CEAED8D0EF53}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="Não Executado"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23350337-5714-4CB9-AE0A-F85FE5C99EC3}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.88671875" customWidth="1"/>
     <col min="4" max="4" width="19.21875" customWidth="1"/>
-    <col min="5" max="5" width="26.5546875" customWidth="1"/>
-    <col min="6" max="6" width="17.44140625" customWidth="1"/>
+    <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.109375" customWidth="1"/>
-    <col min="8" max="8" width="24" customWidth="1"/>
-    <col min="9" max="9" width="11.109375" customWidth="1"/>
-    <col min="10" max="10" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>11</v>
       </c>
@@ -2680,31 +2686,28 @@
         <v>12</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>13</v>
+        <v>59</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>6</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>14</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="I1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="J1" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="6">
         <v>0.41666666666666669</v>
       </c>
@@ -2715,7 +2718,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="8">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="E2" s="8">
         <v>0</v>
@@ -2729,30 +2732,42 @@
       <c r="H2" s="8">
         <v>0</v>
       </c>
-      <c r="I2" s="8">
-        <v>0</v>
-      </c>
-      <c r="J2" s="9">
-        <f>C2+D2+E2+F2+G2+H2+I2</f>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="6"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="9">
-        <f t="shared" ref="J3:J6" si="0">C3+D3+E3+F3+G3+H3+I3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I2" s="9">
+        <f>C2+D2+E2+F2+G2+H2</f>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="6">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="B3" s="7">
+        <v>46252</v>
+      </c>
+      <c r="C3" s="8">
+        <v>19</v>
+      </c>
+      <c r="D3" s="8">
+        <v>1</v>
+      </c>
+      <c r="E3" s="8">
+        <v>8</v>
+      </c>
+      <c r="F3" s="8">
+        <v>6</v>
+      </c>
+      <c r="G3" s="8">
+        <v>8</v>
+      </c>
+      <c r="H3" s="8">
+        <v>1</v>
+      </c>
+      <c r="I3" s="9">
+        <f>C3+D3+E3+F3+G3+H3</f>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="6"/>
       <c r="B4" s="7"/>
       <c r="C4" s="8"/>
@@ -2761,13 +2776,12 @@
       <c r="F4" s="8"/>
       <c r="G4" s="8"/>
       <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="9">
-        <f t="shared" si="0"/>
+      <c r="I4" s="9">
+        <f>C4+D4+E4+F4+G4</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="6"/>
       <c r="B5" s="7"/>
       <c r="C5" s="8"/>
@@ -2776,13 +2790,12 @@
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
       <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="9">
-        <f t="shared" si="0"/>
+      <c r="I5" s="9">
+        <f>C5+D5+E5+F5+G5+H5</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="6"/>
       <c r="B6" s="10"/>
       <c r="C6" s="8"/>
@@ -2791,9 +2804,8 @@
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="9">
-        <f t="shared" si="0"/>
+      <c r="I6" s="9">
+        <f>C6+D6+E6+F6+G6+H6</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dados - 13/08/2026 16:30
</commit_message>
<xml_diff>
--- a/pat/PAT.xlsx
+++ b/pat/PAT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\pat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A835902-C72A-4FE4-9EC6-0E149FC08DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39633080-0074-4468-AF1B-9A66FEA34469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenarios_hml" sheetId="1" r:id="rId1"/>
@@ -1288,9 +1288,6 @@
     <t>Em Teste</t>
   </si>
   <si>
-    <t>Disponivel para reteste</t>
-  </si>
-  <si>
     <t>Não Liberado</t>
   </si>
   <si>
@@ -1301,6 +1298,9 @@
   </si>
   <si>
     <t>Aprovados</t>
+  </si>
+  <si>
+    <t>Ag Reteste</t>
   </si>
 </sst>
 </file>
@@ -1359,7 +1359,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1414,6 +1414,12 @@
         <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -1456,7 +1462,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1530,9 +1536,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1545,9 +1548,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1556,6 +1556,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1892,7 +1895,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3CBE49E-44A1-44E6-BD58-CEAED8D0EF53}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:E44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1920,14 +1922,14 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A2" s="19">
         <v>1</v>
       </c>
       <c r="B2" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="30" t="s">
         <v>17</v>
       </c>
       <c r="D2" s="19" t="s">
@@ -1937,31 +1939,31 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="22">
+    <row r="3" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="19">
         <v>2</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="C3" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="22" t="s">
+      <c r="D3" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="19" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="19">
         <v>3</v>
       </c>
       <c r="B4" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="31" t="s">
+      <c r="C4" s="30" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="19" t="s">
@@ -1971,31 +1973,31 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="24">
+    <row r="5" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A5" s="19">
         <v>4</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="20" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="E5" s="24" t="s">
+      <c r="D5" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" s="19" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A6" s="24">
         <v>5</v>
       </c>
       <c r="B6" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="29" t="s">
         <v>21</v>
       </c>
       <c r="D6" s="24" t="s">
@@ -2005,14 +2007,14 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A7" s="19">
         <v>6</v>
       </c>
       <c r="B7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="31" t="s">
+      <c r="C7" s="30" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="19" t="s">
@@ -2022,14 +2024,14 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="24">
         <v>7</v>
       </c>
       <c r="B8" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="33" t="s">
+      <c r="C8" s="31" t="s">
         <v>23</v>
       </c>
       <c r="D8" s="24" t="s">
@@ -2040,23 +2042,23 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="3">
+      <c r="A9" s="24">
         <v>8</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="3" t="s">
+      <c r="D9" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" s="24" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="24">
         <v>9</v>
       </c>
@@ -2073,14 +2075,14 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="19">
         <v>10</v>
       </c>
       <c r="B11" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="29" t="s">
+      <c r="C11" s="28" t="s">
         <v>26</v>
       </c>
       <c r="D11" s="19" t="s">
@@ -2090,7 +2092,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="19">
         <v>11</v>
       </c>
@@ -2107,7 +2109,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -2118,13 +2120,13 @@
         <v>28</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -2135,13 +2137,13 @@
         <v>29</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="19">
         <v>14</v>
       </c>
@@ -2158,24 +2160,24 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="24">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="19">
         <v>15</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="20" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="E16" s="24" t="s">
+      <c r="D16" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E16" s="19" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -2186,13 +2188,13 @@
         <v>3</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -2203,20 +2205,20 @@
         <v>4</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="24">
         <v>18</v>
       </c>
       <c r="B19" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="34" t="s">
+      <c r="C19" s="32" t="s">
         <v>5</v>
       </c>
       <c r="D19" s="24" t="s">
@@ -2226,7 +2228,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -2237,13 +2239,13 @@
         <v>31</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -2254,13 +2256,13 @@
         <v>32</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -2271,13 +2273,13 @@
         <v>33</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -2288,13 +2290,13 @@
         <v>34</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A24" s="24">
         <v>23</v>
       </c>
@@ -2311,14 +2313,14 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25" s="19">
         <v>24</v>
       </c>
       <c r="B25" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="29" t="s">
+      <c r="C25" s="28" t="s">
         <v>36</v>
       </c>
       <c r="D25" s="19" t="s">
@@ -2328,14 +2330,14 @@
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="19">
         <v>25</v>
       </c>
       <c r="B26" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="C26" s="29" t="s">
+      <c r="C26" s="28" t="s">
         <v>37</v>
       </c>
       <c r="D26" s="19" t="s">
@@ -2345,41 +2347,41 @@
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="22">
+    <row r="27" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A27" s="24">
         <v>26</v>
       </c>
-      <c r="B27" s="23" t="s">
+      <c r="B27" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C27" s="27" t="s">
+      <c r="C27" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="D27" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="E27" s="22" t="s">
+      <c r="D27" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="E27" s="24" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="22">
+    <row r="28" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="24">
         <v>27</v>
       </c>
-      <c r="B28" s="23" t="s">
+      <c r="B28" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C28" s="27" t="s">
+      <c r="C28" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="D28" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="E28" s="22" t="s">
+      <c r="D28" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="E28" s="24" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A29" s="24">
         <v>28</v>
       </c>
@@ -2396,7 +2398,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -2407,13 +2409,13 @@
         <v>3</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -2424,13 +2426,13 @@
         <v>3</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -2441,54 +2443,54 @@
         <v>40</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="26.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="22">
+    <row r="33" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="24">
         <v>32</v>
       </c>
-      <c r="B33" s="23" t="s">
+      <c r="B33" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C33" s="28" t="s">
+      <c r="C33" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="D33" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="E33" s="22" t="s">
+      <c r="D33" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="E33" s="24" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="22">
+    <row r="34" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="24">
         <v>33</v>
       </c>
-      <c r="B34" s="23" t="s">
+      <c r="B34" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="C34" s="28" t="s">
+      <c r="C34" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="D34" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="E34" s="22" t="s">
+      <c r="D34" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="E34" s="24" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="52.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A35" s="22">
         <v>34</v>
       </c>
       <c r="B35" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C35" s="28" t="s">
+      <c r="C35" s="27" t="s">
         <v>42</v>
       </c>
       <c r="D35" s="22" t="s">
@@ -2498,7 +2500,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -2509,13 +2511,13 @@
         <v>43</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -2526,20 +2528,20 @@
         <v>39</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A38" s="24">
         <v>37</v>
       </c>
       <c r="B38" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="C38" s="35" t="s">
+      <c r="C38" s="33" t="s">
         <v>44</v>
       </c>
       <c r="D38" s="24" t="s">
@@ -2549,7 +2551,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -2560,13 +2562,13 @@
         <v>3</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -2577,13 +2579,13 @@
         <v>45</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -2594,13 +2596,13 @@
         <v>46</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -2611,13 +2613,13 @@
         <v>47</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -2628,13 +2630,13 @@
         <v>48</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -2645,20 +2647,14 @@
         <v>49</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>51</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E44" xr:uid="{A3CBE49E-44A1-44E6-BD58-CEAED8D0EF53}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="Não Executado"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:E44" xr:uid="{A3CBE49E-44A1-44E6-BD58-CEAED8D0EF53}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
@@ -2686,19 +2682,19 @@
         <v>12</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>6</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>13</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>14</v>
@@ -2739,7 +2735,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="6">
-        <v>0.41666666666666669</v>
+        <v>0.6875</v>
       </c>
       <c r="B3" s="7">
         <v>46252</v>
@@ -2748,19 +2744,19 @@
         <v>19</v>
       </c>
       <c r="D3" s="8">
+        <v>0</v>
+      </c>
+      <c r="E3" s="8">
+        <v>11</v>
+      </c>
+      <c r="F3" s="8">
         <v>1</v>
       </c>
-      <c r="E3" s="8">
-        <v>8</v>
-      </c>
-      <c r="F3" s="8">
-        <v>6</v>
-      </c>
       <c r="G3" s="8">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H3" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I3" s="9">
         <f>C3+D3+E3+F3+G3+H3</f>

</xml_diff>

<commit_message>
Atualiza dados - 13/08/2026 16:36
</commit_message>
<xml_diff>
--- a/pat/PAT.xlsx
+++ b/pat/PAT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\pat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39633080-0074-4468-AF1B-9A66FEA34469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{922C5926-7B30-48AC-AEB7-C13042ED11CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenarios_hml" sheetId="1" r:id="rId1"/>
@@ -2738,7 +2738,7 @@
         <v>0.6875</v>
       </c>
       <c r="B3" s="7">
-        <v>46252</v>
+        <v>46247</v>
       </c>
       <c r="C3" s="8">
         <v>19</v>

</xml_diff>

<commit_message>
Atualiza dados - 14/08/2026 12:01
</commit_message>
<xml_diff>
--- a/pat/PAT.xlsx
+++ b/pat/PAT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\pat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{752993CF-852B-464D-B46A-54710BECC69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6B7ADD6-FE56-4131-A27D-06D9DF0C5F6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
   </bookViews>
@@ -920,7 +920,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -969,6 +969,12 @@
         <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -1011,7 +1017,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1055,31 +1061,28 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1452,7 +1455,7 @@
       <c r="B2" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="19" t="s">
         <v>15</v>
       </c>
       <c r="D2" s="10" t="s">
@@ -1469,7 +1472,7 @@
       <c r="B3" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="19" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="10" t="s">
@@ -1486,7 +1489,7 @@
       <c r="B4" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="19" t="s">
         <v>17</v>
       </c>
       <c r="D4" s="10" t="s">
@@ -1503,7 +1506,7 @@
       <c r="B5" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="19" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="10" t="s">
@@ -1514,19 +1517,19 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="15">
+      <c r="A6" s="10">
         <v>5</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" s="15" t="s">
+      <c r="D6" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1537,7 +1540,7 @@
       <c r="B7" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="19" t="s">
         <v>20</v>
       </c>
       <c r="D7" s="10" t="s">
@@ -1548,53 +1551,53 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="15">
+      <c r="A8" s="10">
         <v>7</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="11" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" s="15" t="s">
+      <c r="D8" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="10" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="15">
+      <c r="A9" s="10">
         <v>8</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9" s="15" t="s">
+      <c r="D9" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="15">
+      <c r="A10" s="10">
         <v>9</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E10" s="15" t="s">
+      <c r="D10" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1605,7 +1608,7 @@
       <c r="B11" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>24</v>
       </c>
       <c r="D11" s="10" t="s">
@@ -1656,7 +1659,7 @@
       <c r="B14" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D14" s="10" t="s">
@@ -1667,36 +1670,36 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="15">
+      <c r="A15" s="10">
         <v>18</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="11" t="s">
         <v>6</v>
       </c>
       <c r="C15" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="D15" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E15" s="15" t="s">
+      <c r="D15" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="15">
+      <c r="A16" s="10">
         <v>23</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="C16" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D16" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E16" s="15" t="s">
+      <c r="D16" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1707,7 +1710,7 @@
       <c r="B17" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C17" s="18" t="s">
         <v>28</v>
       </c>
       <c r="D17" s="10" t="s">
@@ -1724,7 +1727,7 @@
       <c r="B18" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="18" t="s">
         <v>29</v>
       </c>
       <c r="D18" s="10" t="s">
@@ -1735,36 +1738,36 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="15">
+      <c r="A19" s="10">
         <v>28</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E19" s="15" t="s">
+      <c r="D19" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" s="10" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="15">
+      <c r="A20" s="10">
         <v>32</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="25" t="s">
+      <c r="C20" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="D20" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E20" s="15" t="s">
+      <c r="D20" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" s="10" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1775,7 +1778,7 @@
       <c r="B21" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="25" t="s">
+      <c r="C21" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D21" s="15" t="s">
@@ -1792,7 +1795,7 @@
       <c r="B22" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="17" t="s">
         <v>31</v>
       </c>
       <c r="D22" s="13" t="s">
@@ -1809,7 +1812,7 @@
       <c r="B23" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="C23" s="24" t="s">
+      <c r="C23" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D23" s="15" t="s">

</xml_diff>

<commit_message>
Atualiza dados - 14/08/2026 12:29
</commit_message>
<xml_diff>
--- a/pat/PAT.xlsx
+++ b/pat/PAT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\pat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6B7ADD6-FE56-4131-A27D-06D9DF0C5F6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{859BD1AF-44BB-4418-9F90-00094FD084EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenarios_hml" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="42">
   <si>
     <t>Número do cenário</t>
   </si>
@@ -862,6 +862,9 @@
   </si>
   <si>
     <t>Aprovados</t>
+  </si>
+  <si>
+    <t>Ag Corração</t>
   </si>
 </sst>
 </file>
@@ -1844,9 +1847,9 @@
     <col min="3" max="3" width="17.88671875" customWidth="1"/>
     <col min="4" max="4" width="19.21875" customWidth="1"/>
     <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" customWidth="1"/>
     <col min="7" max="7" width="19.109375" customWidth="1"/>
-    <col min="8" max="8" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.77734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="5.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1867,7 +1870,7 @@
         <v>40</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>38</v>
@@ -1940,17 +1943,33 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
+      <c r="A4" s="5">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="B4" s="6">
+        <v>46248</v>
+      </c>
+      <c r="C4" s="7">
+        <v>0</v>
+      </c>
+      <c r="D4" s="7">
+        <v>0</v>
+      </c>
+      <c r="E4" s="7">
+        <v>19</v>
+      </c>
+      <c r="F4" s="7">
+        <v>3</v>
+      </c>
+      <c r="G4" s="7">
+        <v>0</v>
+      </c>
+      <c r="H4" s="7">
+        <v>0</v>
+      </c>
       <c r="I4" s="8">
         <f>C4+D4+E4+F4+G4</f>
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza dados - 14/08/2026 12:31
</commit_message>
<xml_diff>
--- a/pat/PAT.xlsx
+++ b/pat/PAT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\pat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{859BD1AF-44BB-4418-9F90-00094FD084EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC445DC5-B27C-4AFB-B532-C3A3AA5DD24C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{D147479C-2CBD-48F2-8B80-85CBDC094C22}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="40">
   <si>
     <t>Número do cenário</t>
   </si>
@@ -79,9 +79,6 @@
   </si>
   <si>
     <t>Reprovado</t>
-  </si>
-  <si>
-    <t>Disponível para reteste</t>
   </si>
   <si>
     <t>Total</t>
@@ -856,9 +853,6 @@
   </si>
   <si>
     <t>Em Execução</t>
-  </si>
-  <si>
-    <t>Não Liberados</t>
   </si>
   <si>
     <t>Aprovados</t>
@@ -1020,7 +1014,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1042,7 +1036,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1445,384 +1438,384 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="10">
-        <v>1</v>
-      </c>
-      <c r="B2" s="11" t="s">
+      <c r="E2" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D3" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="9">
+        <v>5</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="9">
+        <v>6</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="9">
+        <v>7</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="9">
+        <v>9</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="9">
+        <v>10</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="9">
+        <v>11</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="9">
+        <v>14</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="9">
+        <v>15</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="9">
+        <v>18</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="9">
+        <v>23</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="9">
+        <v>24</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="9">
+        <v>25</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="9">
+        <v>28</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="9">
+        <v>32</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="14">
+        <v>33</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E21" s="14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="12">
         <v>34</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="10">
-        <v>2</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="10" t="s">
+      <c r="B22" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="14">
+        <v>37</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="10">
-        <v>3</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="10">
-        <v>4</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="10">
-        <v>5</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="10">
-        <v>6</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="10">
-        <v>7</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="10">
-        <v>8</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="10">
-        <v>9</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="10">
-        <v>10</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="10">
-        <v>11</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10">
-        <v>14</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="10">
-        <v>15</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="10">
-        <v>18</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="10">
-        <v>23</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="10">
-        <v>24</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="10">
-        <v>25</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C18" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="10">
-        <v>28</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="10">
-        <v>32</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C20" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="15">
-        <v>33</v>
-      </c>
-      <c r="B21" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="13">
-        <v>34</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="D22" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="15">
-        <v>37</v>
-      </c>
-      <c r="B23" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="20" t="s">
-        <v>32</v>
-      </c>
-      <c r="D23" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>34</v>
+      <c r="E23" s="14" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1840,20 +1833,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23350337-5714-4CB9-AE0A-F85FE5C99EC3}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.88671875" customWidth="1"/>
-    <col min="4" max="4" width="19.21875" customWidth="1"/>
-    <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" customWidth="1"/>
-    <col min="7" max="7" width="19.109375" customWidth="1"/>
-    <col min="8" max="8" width="21.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.21875" customWidth="1"/>
+    <col min="4" max="4" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="19.109375" customWidth="1"/>
+    <col min="7" max="7" width="5.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>9</v>
       </c>
@@ -1861,28 +1852,22 @@
         <v>10</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>40</v>
-      </c>
       <c r="F1" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="5">
         <v>0.41666666666666669</v>
       </c>
@@ -1890,10 +1875,10 @@
         <v>46244</v>
       </c>
       <c r="C2" s="7">
+        <v>43</v>
+      </c>
+      <c r="D2" s="7">
         <v>0</v>
-      </c>
-      <c r="D2" s="7">
-        <v>43</v>
       </c>
       <c r="E2" s="7">
         <v>0</v>
@@ -1901,18 +1886,12 @@
       <c r="F2" s="7">
         <v>0</v>
       </c>
-      <c r="G2" s="7">
-        <v>0</v>
-      </c>
-      <c r="H2" s="7">
-        <v>0</v>
-      </c>
-      <c r="I2" s="8">
-        <f>C2+D2+E2+F2+G2+H2</f>
+      <c r="G2" s="8">
+        <f>C2+D2+E2+F2</f>
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>0.6875</v>
       </c>
@@ -1920,29 +1899,23 @@
         <v>46247</v>
       </c>
       <c r="C3" s="7">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="D3" s="7">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E3" s="7">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="F3" s="7">
-        <v>1</v>
-      </c>
-      <c r="G3" s="7">
         <v>10</v>
       </c>
-      <c r="H3" s="7">
-        <v>2</v>
-      </c>
-      <c r="I3" s="8">
-        <f>C3+D3+E3+F3+G3+H3</f>
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G3" s="8">
+        <f>C3+D3+E3+F3</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>0.52083333333333337</v>
       </c>
@@ -1953,50 +1926,28 @@
         <v>0</v>
       </c>
       <c r="D4" s="7">
+        <v>19</v>
+      </c>
+      <c r="E4" s="7">
+        <v>3</v>
+      </c>
+      <c r="F4" s="7">
         <v>0</v>
       </c>
-      <c r="E4" s="7">
-        <v>19</v>
-      </c>
-      <c r="F4" s="7">
-        <v>3</v>
-      </c>
-      <c r="G4" s="7">
-        <v>0</v>
-      </c>
-      <c r="H4" s="7">
-        <v>0</v>
-      </c>
-      <c r="I4" s="8">
-        <f>C4+D4+E4+F4+G4</f>
+      <c r="G4" s="8">
+        <f>C4+D4+E4+F4</f>
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="6"/>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="8">
-        <f>C5+D5+E5+F5+G5+H5</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="8">
-        <f>C6+D6+E6+F6+G6+H6</f>
+      <c r="G5" s="8">
+        <f t="shared" ref="G5" si="0">C5+D5+E5+F5</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>